<commit_message>
added carbon data and ran the initial carbon analysis
</commit_message>
<xml_diff>
--- a/data/biomass/Aveiro_grid_info_final.xlsx
+++ b/data/biomass/Aveiro_grid_info_final.xlsx
@@ -22,22 +22,8 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId4"/>
+    <pivotCache cacheId="34" r:id="rId4"/>
   </pivotCaches>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -1541,6 +1527,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Liberation Sans"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1548,6 +1535,7 @@
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Liberation Sans"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1556,18 +1544,21 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Liberation Sans"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Liberation Sans"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Liberation Sans"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1663,7 +1654,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1748,6 +1739,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1963,7 +1957,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="barille-l" refreshedDate="46044.482672569444" createdVersion="8" refreshedVersion="6" minRefreshableVersion="3" recordCount="179">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="barille-l" refreshedDate="46069.626449421296" createdVersion="8" refreshedVersion="6" minRefreshableVersion="3" recordCount="179">
   <cacheSource type="worksheet">
     <worksheetSource ref="B1:E1048576" sheet="seagrass biomass"/>
   </cacheSource>
@@ -3164,7 +3158,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Draaitabel1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Waarden" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Draaitabel1" cacheId="34" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Waarden" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="G1:K93" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -8048,6 +8042,7 @@
         <v>369</v>
       </c>
       <c r="E2" s="2">
+        <f>IFERROR(IF(VLOOKUP(B2,$O$5:$P$148,2)="empty",0,VLOOKUP(B2,$O$5:$P$148,2)),0)</f>
         <v>2797</v>
       </c>
       <c r="G2" s="6" t="s">
@@ -8089,6 +8084,7 @@
         <v>370</v>
       </c>
       <c r="E3" s="2">
+        <f t="shared" ref="E3:E66" si="0">IFERROR(IF(VLOOKUP(B3,$O$5:$P$148,2)="empty",0,VLOOKUP(B3,$O$5:$P$148,2)),0)</f>
         <v>1048</v>
       </c>
       <c r="G3" s="15">
@@ -8125,6 +8121,7 @@
         <v>369</v>
       </c>
       <c r="E4" s="2">
+        <f t="shared" si="0"/>
         <v>1876</v>
       </c>
       <c r="G4" s="2">
@@ -8163,6 +8160,7 @@
         <v>370</v>
       </c>
       <c r="E5" s="2">
+        <f t="shared" si="0"/>
         <v>608</v>
       </c>
       <c r="G5" s="2">
@@ -8203,7 +8201,7 @@
         <v>369</v>
       </c>
       <c r="E6" s="2">
-        <f>3982-6.2</f>
+        <f t="shared" si="0"/>
         <v>3975.8</v>
       </c>
       <c r="G6" s="2">
@@ -8242,6 +8240,7 @@
         <v>370</v>
       </c>
       <c r="E7" s="2">
+        <f t="shared" si="0"/>
         <v>2080</v>
       </c>
       <c r="G7" s="2">
@@ -8280,6 +8279,7 @@
         <v>369</v>
       </c>
       <c r="E8" s="2">
+        <f t="shared" si="0"/>
         <v>3531</v>
       </c>
       <c r="G8" s="2">
@@ -8318,6 +8318,7 @@
         <v>370</v>
       </c>
       <c r="E9" s="2">
+        <f t="shared" si="0"/>
         <v>2364</v>
       </c>
       <c r="G9" s="2">
@@ -8357,6 +8358,7 @@
         <v>369</v>
       </c>
       <c r="E10" s="2">
+        <f t="shared" si="0"/>
         <v>750</v>
       </c>
       <c r="G10" s="2">
@@ -8395,6 +8397,7 @@
         <v>370</v>
       </c>
       <c r="E11" s="2">
+        <f t="shared" si="0"/>
         <v>345</v>
       </c>
       <c r="G11" s="2">
@@ -8433,6 +8436,7 @@
         <v>369</v>
       </c>
       <c r="E12" s="2">
+        <f t="shared" si="0"/>
         <v>754</v>
       </c>
       <c r="G12" s="2">
@@ -8471,6 +8475,7 @@
         <v>370</v>
       </c>
       <c r="E13" s="2">
+        <f t="shared" si="0"/>
         <v>582</v>
       </c>
       <c r="G13" s="2">
@@ -8509,6 +8514,7 @@
         <v>369</v>
       </c>
       <c r="E14" s="2">
+        <f t="shared" si="0"/>
         <v>3628</v>
       </c>
       <c r="G14" s="2">
@@ -8547,6 +8553,7 @@
         <v>370</v>
       </c>
       <c r="E15" s="2">
+        <f t="shared" si="0"/>
         <v>977</v>
       </c>
       <c r="G15" s="2">
@@ -8585,6 +8592,7 @@
         <v>369</v>
       </c>
       <c r="E16" s="2">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="G16" s="2">
@@ -8623,6 +8631,7 @@
         <v>370</v>
       </c>
       <c r="E17" s="2">
+        <f t="shared" si="0"/>
         <v>118</v>
       </c>
       <c r="G17" s="2">
@@ -8659,6 +8668,7 @@
         <v>369</v>
       </c>
       <c r="E18" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G18" s="2">
@@ -8695,6 +8705,7 @@
         <v>370</v>
       </c>
       <c r="E19" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G19" s="2">
@@ -8731,6 +8742,7 @@
         <v>369</v>
       </c>
       <c r="E20" s="2">
+        <f t="shared" si="0"/>
         <v>2650</v>
       </c>
       <c r="G20" s="2">
@@ -8767,6 +8779,7 @@
         <v>370</v>
       </c>
       <c r="E21" s="2">
+        <f t="shared" si="0"/>
         <v>1147</v>
       </c>
       <c r="G21" s="2">
@@ -8803,6 +8816,7 @@
         <v>369</v>
       </c>
       <c r="E22" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G22" s="2">
@@ -8839,6 +8853,7 @@
         <v>370</v>
       </c>
       <c r="E23" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G23" s="15">
@@ -8875,6 +8890,7 @@
         <v>369</v>
       </c>
       <c r="E24" s="2">
+        <f t="shared" si="0"/>
         <v>2564</v>
       </c>
       <c r="G24" s="2">
@@ -8911,6 +8927,7 @@
         <v>370</v>
       </c>
       <c r="E25" s="2">
+        <f t="shared" si="0"/>
         <v>2102</v>
       </c>
       <c r="G25" s="2">
@@ -8947,6 +8964,7 @@
         <v>369</v>
       </c>
       <c r="E26" s="2">
+        <f t="shared" si="0"/>
         <v>1891</v>
       </c>
       <c r="G26" s="2">
@@ -8983,6 +9001,7 @@
         <v>370</v>
       </c>
       <c r="E27" s="2">
+        <f t="shared" si="0"/>
         <v>891</v>
       </c>
       <c r="G27" s="2">
@@ -9019,6 +9038,7 @@
         <v>369</v>
       </c>
       <c r="E28" s="2">
+        <f t="shared" si="0"/>
         <v>2057</v>
       </c>
       <c r="G28" s="2">
@@ -9055,6 +9075,7 @@
         <v>370</v>
       </c>
       <c r="E29" s="2">
+        <f t="shared" si="0"/>
         <v>1686</v>
       </c>
       <c r="G29" s="2">
@@ -9091,6 +9112,7 @@
         <v>369</v>
       </c>
       <c r="E30" s="2">
+        <f t="shared" si="0"/>
         <v>926</v>
       </c>
       <c r="G30" s="2">
@@ -9127,6 +9149,7 @@
         <v>370</v>
       </c>
       <c r="E31" s="2">
+        <f t="shared" si="0"/>
         <v>1187</v>
       </c>
       <c r="G31" s="2">
@@ -9163,6 +9186,7 @@
         <v>369</v>
       </c>
       <c r="E32" s="2">
+        <f t="shared" si="0"/>
         <v>2434</v>
       </c>
       <c r="G32" s="2">
@@ -9199,6 +9223,7 @@
         <v>370</v>
       </c>
       <c r="E33" s="2">
+        <f t="shared" si="0"/>
         <v>1076</v>
       </c>
       <c r="G33" s="2">
@@ -9235,6 +9260,7 @@
         <v>369</v>
       </c>
       <c r="E34" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G34" s="2">
@@ -9271,6 +9297,7 @@
         <v>370</v>
       </c>
       <c r="E35" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G35" s="2">
@@ -9307,6 +9334,7 @@
         <v>369</v>
       </c>
       <c r="E36" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G36" s="2">
@@ -9343,6 +9371,7 @@
         <v>370</v>
       </c>
       <c r="E37" s="2">
+        <f t="shared" si="0"/>
         <v>125</v>
       </c>
       <c r="G37" s="2">
@@ -9379,6 +9408,7 @@
         <v>369</v>
       </c>
       <c r="E38" s="2">
+        <f t="shared" si="0"/>
         <v>821</v>
       </c>
       <c r="G38" s="2">
@@ -9415,6 +9445,7 @@
         <v>370</v>
       </c>
       <c r="E39" s="2">
+        <f t="shared" si="0"/>
         <v>561</v>
       </c>
       <c r="G39" s="2">
@@ -9451,6 +9482,7 @@
         <v>369</v>
       </c>
       <c r="E40" s="2">
+        <f t="shared" si="0"/>
         <v>951</v>
       </c>
       <c r="G40" s="2">
@@ -9487,7 +9519,7 @@
         <v>370</v>
       </c>
       <c r="E41" s="2">
-        <f>578-4.5</f>
+        <f t="shared" si="0"/>
         <v>573.5</v>
       </c>
       <c r="G41" s="2">
@@ -9524,6 +9556,7 @@
         <v>369</v>
       </c>
       <c r="E42" s="2">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="G42" s="2">
@@ -9560,6 +9593,7 @@
         <v>370</v>
       </c>
       <c r="E43" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G43" s="2">
@@ -9596,6 +9630,7 @@
         <v>369</v>
       </c>
       <c r="E44" s="2">
+        <f t="shared" si="0"/>
         <v>1476</v>
       </c>
       <c r="G44" s="2">
@@ -9633,6 +9668,7 @@
         <v>370</v>
       </c>
       <c r="E45" s="2">
+        <f t="shared" si="0"/>
         <v>1194</v>
       </c>
       <c r="G45" s="2">
@@ -9669,6 +9705,7 @@
         <v>369</v>
       </c>
       <c r="E46" s="2">
+        <f t="shared" si="0"/>
         <v>1220</v>
       </c>
       <c r="G46" s="2">
@@ -9705,6 +9742,7 @@
         <v>370</v>
       </c>
       <c r="E47" s="2">
+        <f t="shared" si="0"/>
         <v>2529</v>
       </c>
       <c r="G47" s="2">
@@ -9741,6 +9779,7 @@
         <v>369</v>
       </c>
       <c r="E48" s="2">
+        <f t="shared" si="0"/>
         <v>1701</v>
       </c>
       <c r="G48" s="2">
@@ -9777,6 +9816,7 @@
         <v>370</v>
       </c>
       <c r="E49" s="2">
+        <f t="shared" si="0"/>
         <v>1821</v>
       </c>
       <c r="G49" s="2">
@@ -9813,6 +9853,7 @@
         <v>369</v>
       </c>
       <c r="E50" s="2">
+        <f t="shared" si="0"/>
         <v>1415</v>
       </c>
       <c r="G50" s="2">
@@ -9849,6 +9890,7 @@
         <v>370</v>
       </c>
       <c r="E51" s="2">
+        <f t="shared" si="0"/>
         <v>833</v>
       </c>
       <c r="G51" s="2">
@@ -9885,6 +9927,7 @@
         <v>369</v>
       </c>
       <c r="E52" s="2">
+        <f t="shared" si="0"/>
         <v>1552</v>
       </c>
       <c r="G52" s="2">
@@ -9921,6 +9964,7 @@
         <v>370</v>
       </c>
       <c r="E53" s="2">
+        <f t="shared" si="0"/>
         <v>561</v>
       </c>
       <c r="G53" s="2">
@@ -9957,6 +10001,7 @@
         <v>369</v>
       </c>
       <c r="E54" s="2">
+        <f t="shared" si="0"/>
         <v>2799</v>
       </c>
       <c r="G54" s="2">
@@ -9993,6 +10038,7 @@
         <v>370</v>
       </c>
       <c r="E55" s="2">
+        <f t="shared" si="0"/>
         <v>1299</v>
       </c>
       <c r="G55" s="2">
@@ -10029,6 +10075,7 @@
         <v>369</v>
       </c>
       <c r="E56" s="2">
+        <f t="shared" si="0"/>
         <v>392</v>
       </c>
       <c r="G56" s="2">
@@ -10065,6 +10112,7 @@
         <v>370</v>
       </c>
       <c r="E57" s="2">
+        <f t="shared" si="0"/>
         <v>156</v>
       </c>
       <c r="G57" s="2">
@@ -10101,6 +10149,7 @@
         <v>369</v>
       </c>
       <c r="E58" s="2">
+        <f t="shared" si="0"/>
         <v>465</v>
       </c>
       <c r="G58" s="2">
@@ -10137,6 +10186,7 @@
         <v>370</v>
       </c>
       <c r="E59" s="2">
+        <f t="shared" si="0"/>
         <v>1025</v>
       </c>
       <c r="G59" s="2">
@@ -10173,6 +10223,7 @@
         <v>369</v>
       </c>
       <c r="E60" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G60" s="2">
@@ -10209,6 +10260,7 @@
         <v>370</v>
       </c>
       <c r="E61" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G61" s="2">
@@ -10245,6 +10297,7 @@
         <v>369</v>
       </c>
       <c r="E62" s="2">
+        <f t="shared" si="0"/>
         <v>931</v>
       </c>
       <c r="G62" s="2">
@@ -10281,6 +10334,7 @@
         <v>370</v>
       </c>
       <c r="E63" s="2">
+        <f t="shared" si="0"/>
         <v>712</v>
       </c>
       <c r="G63" s="2">
@@ -10317,6 +10371,7 @@
         <v>369</v>
       </c>
       <c r="E64" s="2">
+        <f t="shared" si="0"/>
         <v>510</v>
       </c>
       <c r="G64" s="2">
@@ -10353,6 +10408,7 @@
         <v>370</v>
       </c>
       <c r="E65" s="2">
+        <f t="shared" si="0"/>
         <v>557</v>
       </c>
       <c r="G65" s="2">
@@ -10389,6 +10445,7 @@
         <v>369</v>
       </c>
       <c r="E66" s="2">
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="G66" s="2">
@@ -10425,6 +10482,7 @@
         <v>370</v>
       </c>
       <c r="E67" s="2">
+        <f t="shared" ref="E67:E130" si="1">IFERROR(IF(VLOOKUP(B67,$O$5:$P$148,2)="empty",0,VLOOKUP(B67,$O$5:$P$148,2)),0)</f>
         <v>189</v>
       </c>
       <c r="G67" s="2">
@@ -10461,7 +10519,7 @@
         <v>369</v>
       </c>
       <c r="E68" s="2">
-        <f>977-106</f>
+        <f t="shared" si="1"/>
         <v>871</v>
       </c>
       <c r="G68" s="2">
@@ -10498,6 +10556,7 @@
         <v>370</v>
       </c>
       <c r="E69" s="2">
+        <f t="shared" si="1"/>
         <v>401</v>
       </c>
       <c r="G69" s="2">
@@ -10534,6 +10593,7 @@
         <v>369</v>
       </c>
       <c r="E70" s="2">
+        <f t="shared" si="1"/>
         <v>994</v>
       </c>
       <c r="G70" s="2">
@@ -10570,6 +10630,7 @@
         <v>370</v>
       </c>
       <c r="E71" s="2">
+        <f t="shared" si="1"/>
         <v>343</v>
       </c>
       <c r="G71" s="2">
@@ -10607,6 +10668,7 @@
         <v>369</v>
       </c>
       <c r="E72" s="2">
+        <f t="shared" si="1"/>
         <v>2523</v>
       </c>
       <c r="G72" s="2">
@@ -10643,6 +10705,7 @@
         <v>370</v>
       </c>
       <c r="E73" s="2">
+        <f t="shared" si="1"/>
         <v>1219</v>
       </c>
       <c r="G73" s="2">
@@ -10679,6 +10742,7 @@
         <v>369</v>
       </c>
       <c r="E74" s="2">
+        <f t="shared" si="1"/>
         <v>2695</v>
       </c>
       <c r="G74" s="2">
@@ -10715,6 +10779,7 @@
         <v>370</v>
       </c>
       <c r="E75" s="2">
+        <f t="shared" si="1"/>
         <v>1160</v>
       </c>
       <c r="G75" s="2" t="s">
@@ -10745,6 +10810,7 @@
         <v>369</v>
       </c>
       <c r="E76" s="2">
+        <f t="shared" si="1"/>
         <v>933</v>
       </c>
       <c r="G76" s="2">
@@ -10781,6 +10847,7 @@
         <v>370</v>
       </c>
       <c r="E77" s="2">
+        <f t="shared" si="1"/>
         <v>750</v>
       </c>
       <c r="G77" s="2">
@@ -10817,6 +10884,7 @@
         <v>369</v>
       </c>
       <c r="E78" s="2">
+        <f t="shared" si="1"/>
         <v>85</v>
       </c>
       <c r="G78" s="2">
@@ -10853,6 +10921,7 @@
         <v>370</v>
       </c>
       <c r="E79" s="2">
+        <f t="shared" si="1"/>
         <v>719</v>
       </c>
       <c r="G79" s="2">
@@ -10889,6 +10958,7 @@
         <v>369</v>
       </c>
       <c r="E80" s="2">
+        <f t="shared" si="1"/>
         <v>2790</v>
       </c>
       <c r="G80" s="2">
@@ -10925,6 +10995,7 @@
         <v>370</v>
       </c>
       <c r="E81" s="2">
+        <f t="shared" si="1"/>
         <v>888</v>
       </c>
       <c r="G81" s="2">
@@ -10961,6 +11032,7 @@
         <v>369</v>
       </c>
       <c r="E82" s="2">
+        <f t="shared" si="1"/>
         <v>2113</v>
       </c>
       <c r="G82" s="2">
@@ -10997,6 +11069,7 @@
         <v>370</v>
       </c>
       <c r="E83" s="2">
+        <f t="shared" si="1"/>
         <v>675</v>
       </c>
       <c r="G83" s="2">
@@ -11033,7 +11106,7 @@
         <v>369</v>
       </c>
       <c r="E84" s="2">
-        <f>2237-66</f>
+        <f t="shared" si="1"/>
         <v>2171</v>
       </c>
       <c r="G84" s="2">
@@ -11070,7 +11143,7 @@
         <v>370</v>
       </c>
       <c r="E85" s="2">
-        <f>951-18</f>
+        <f t="shared" si="1"/>
         <v>933</v>
       </c>
       <c r="G85" s="2">
@@ -11107,6 +11180,7 @@
         <v>369</v>
       </c>
       <c r="E86" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G86" s="2">
@@ -11143,6 +11217,7 @@
         <v>370</v>
       </c>
       <c r="E87" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G87" s="2">
@@ -11180,6 +11255,7 @@
         <v>369</v>
       </c>
       <c r="E88" s="2">
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="G88" s="2">
@@ -11217,6 +11293,7 @@
         <v>370</v>
       </c>
       <c r="E89" s="2">
+        <f t="shared" si="1"/>
         <v>161</v>
       </c>
       <c r="G89" s="2">
@@ -11253,6 +11330,7 @@
         <v>369</v>
       </c>
       <c r="E90" s="2">
+        <f t="shared" si="1"/>
         <v>2715</v>
       </c>
       <c r="G90" s="2">
@@ -11289,6 +11367,7 @@
         <v>370</v>
       </c>
       <c r="E91" s="2">
+        <f t="shared" si="1"/>
         <v>1696</v>
       </c>
       <c r="G91" s="2">
@@ -11325,6 +11404,7 @@
         <v>369</v>
       </c>
       <c r="E92" s="2">
+        <f t="shared" si="1"/>
         <v>1294</v>
       </c>
       <c r="G92" s="2">
@@ -11361,6 +11441,7 @@
         <v>370</v>
       </c>
       <c r="E93" s="2">
+        <f t="shared" si="1"/>
         <v>454</v>
       </c>
       <c r="G93" s="2" t="s">
@@ -11397,6 +11478,7 @@
         <v>369</v>
       </c>
       <c r="E94" s="2">
+        <f t="shared" si="1"/>
         <v>228</v>
       </c>
       <c r="O94" s="25" t="s">
@@ -11420,6 +11502,7 @@
         <v>370</v>
       </c>
       <c r="E95" s="2">
+        <f t="shared" si="1"/>
         <v>191</v>
       </c>
       <c r="O95" s="22" t="s">
@@ -11443,6 +11526,7 @@
         <v>369</v>
       </c>
       <c r="E96" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O96" s="22" t="s">
@@ -11466,6 +11550,7 @@
         <v>370</v>
       </c>
       <c r="E97" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O97" s="20" t="s">
@@ -11489,6 +11574,7 @@
         <v>369</v>
       </c>
       <c r="E98" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O98" s="20" t="s">
@@ -11512,6 +11598,7 @@
         <v>370</v>
       </c>
       <c r="E99" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O99" s="20" t="s">
@@ -11535,7 +11622,7 @@
         <v>369</v>
       </c>
       <c r="E100" s="2">
-        <f>209-(2.14+0.84)</f>
+        <f t="shared" si="1"/>
         <v>206.02</v>
       </c>
       <c r="O100" s="20" t="s">
@@ -11559,7 +11646,7 @@
         <v>370</v>
       </c>
       <c r="E101" s="2">
-        <f>248-35.6</f>
+        <f t="shared" si="1"/>
         <v>212.4</v>
       </c>
       <c r="O101" s="19" t="s">
@@ -11583,6 +11670,7 @@
         <v>369</v>
       </c>
       <c r="E102" s="2">
+        <f t="shared" si="1"/>
         <v>645</v>
       </c>
       <c r="O102" s="19" t="s">
@@ -11606,6 +11694,7 @@
         <v>370</v>
       </c>
       <c r="E103" s="2">
+        <f t="shared" si="1"/>
         <v>607</v>
       </c>
       <c r="O103" s="22" t="s">
@@ -11630,6 +11719,7 @@
         <v>369</v>
       </c>
       <c r="E104" s="2">
+        <f t="shared" si="1"/>
         <v>1871</v>
       </c>
       <c r="O104" s="22" t="s">
@@ -11654,6 +11744,7 @@
         <v>370</v>
       </c>
       <c r="E105" s="2">
+        <f t="shared" si="1"/>
         <v>1585</v>
       </c>
       <c r="O105" s="21" t="s">
@@ -11677,6 +11768,7 @@
         <v>369</v>
       </c>
       <c r="E106" s="2">
+        <f t="shared" si="1"/>
         <v>1642</v>
       </c>
       <c r="O106" s="21" t="s">
@@ -11702,6 +11794,7 @@
         <v>370</v>
       </c>
       <c r="E107" s="2">
+        <f t="shared" si="1"/>
         <v>1381</v>
       </c>
       <c r="O107" s="22" t="s">
@@ -11727,6 +11820,7 @@
         <v>369</v>
       </c>
       <c r="E108" s="2">
+        <f t="shared" si="1"/>
         <v>315</v>
       </c>
       <c r="O108" s="22" t="s">
@@ -11752,6 +11846,7 @@
         <v>370</v>
       </c>
       <c r="E109" s="2">
+        <f t="shared" si="1"/>
         <v>250</v>
       </c>
       <c r="O109" s="22" t="s">
@@ -11777,6 +11872,7 @@
         <v>369</v>
       </c>
       <c r="E110" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O110" s="22" t="s">
@@ -11800,6 +11896,7 @@
         <v>370</v>
       </c>
       <c r="E111" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O111" s="20" t="s">
@@ -11823,6 +11920,7 @@
         <v>369</v>
       </c>
       <c r="E112" s="2">
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="O112" s="20" t="s">
@@ -11846,6 +11944,7 @@
         <v>370</v>
       </c>
       <c r="E113" s="2">
+        <f t="shared" si="1"/>
         <v>141</v>
       </c>
       <c r="O113" s="20" t="s">
@@ -11869,6 +11968,7 @@
         <v>369</v>
       </c>
       <c r="E114" s="2">
+        <f t="shared" si="1"/>
         <v>2222</v>
       </c>
       <c r="O114" s="20" t="s">
@@ -11892,6 +11992,7 @@
         <v>370</v>
       </c>
       <c r="E115" s="2">
+        <f t="shared" si="1"/>
         <v>939</v>
       </c>
       <c r="O115" s="20" t="s">
@@ -11915,6 +12016,7 @@
         <v>369</v>
       </c>
       <c r="E116" s="2">
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="O116" s="20" t="s">
@@ -11938,6 +12040,7 @@
         <v>370</v>
       </c>
       <c r="E117" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O117" s="26" t="s">
@@ -11961,6 +12064,7 @@
         <v>369</v>
       </c>
       <c r="E118" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O118" s="26" t="s">
@@ -11984,6 +12088,7 @@
         <v>370</v>
       </c>
       <c r="E119" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O119" s="26" t="s">
@@ -12007,6 +12112,7 @@
         <v>369</v>
       </c>
       <c r="E120" s="2">
+        <f t="shared" si="1"/>
         <v>2745</v>
       </c>
       <c r="O120" s="26" t="s">
@@ -12030,6 +12136,7 @@
         <v>370</v>
       </c>
       <c r="E121" s="2">
+        <f t="shared" si="1"/>
         <v>1244</v>
       </c>
       <c r="O121" s="20" t="s">
@@ -12053,6 +12160,7 @@
         <v>369</v>
       </c>
       <c r="E122" s="2">
+        <f t="shared" si="1"/>
         <v>400</v>
       </c>
       <c r="O122" s="20" t="s">
@@ -12076,6 +12184,7 @@
         <v>370</v>
       </c>
       <c r="E123" s="2">
+        <f t="shared" si="1"/>
         <v>338</v>
       </c>
       <c r="O123" s="22" t="s">
@@ -12099,6 +12208,7 @@
         <v>369</v>
       </c>
       <c r="E124" s="2">
+        <f t="shared" si="1"/>
         <v>1514</v>
       </c>
       <c r="O124" s="22" t="s">
@@ -12122,6 +12232,7 @@
         <v>370</v>
       </c>
       <c r="E125" s="2">
+        <f t="shared" si="1"/>
         <v>556</v>
       </c>
       <c r="O125" s="23" t="s">
@@ -12145,6 +12256,7 @@
         <v>369</v>
       </c>
       <c r="E126" s="2">
+        <f t="shared" si="1"/>
         <v>2566</v>
       </c>
       <c r="O126" s="23" t="s">
@@ -12168,6 +12280,7 @@
         <v>370</v>
       </c>
       <c r="E127" s="2">
+        <f t="shared" si="1"/>
         <v>1512</v>
       </c>
       <c r="O127" s="10" t="s">
@@ -12191,6 +12304,7 @@
         <v>369</v>
       </c>
       <c r="E128" s="2">
+        <f t="shared" si="1"/>
         <v>3538</v>
       </c>
       <c r="O128" s="10" t="s">
@@ -12214,6 +12328,7 @@
         <v>370</v>
       </c>
       <c r="E129" s="2">
+        <f t="shared" si="1"/>
         <v>2263</v>
       </c>
       <c r="O129" s="10" t="s">
@@ -12237,6 +12352,7 @@
         <v>369</v>
       </c>
       <c r="E130" s="2">
+        <f t="shared" si="1"/>
         <v>1780</v>
       </c>
       <c r="O130" s="10" t="s">
@@ -12260,6 +12376,7 @@
         <v>370</v>
       </c>
       <c r="E131" s="2">
+        <f t="shared" ref="E131:E161" si="2">IFERROR(IF(VLOOKUP(B131,$O$5:$P$148,2)="empty",0,VLOOKUP(B131,$O$5:$P$148,2)),0)</f>
         <v>1728</v>
       </c>
       <c r="O131" s="10" t="s">
@@ -12283,6 +12400,7 @@
         <v>369</v>
       </c>
       <c r="E132" s="2">
+        <f t="shared" si="2"/>
         <v>3113</v>
       </c>
       <c r="O132" s="10" t="s">
@@ -12306,6 +12424,7 @@
         <v>370</v>
       </c>
       <c r="E133" s="2">
+        <f t="shared" si="2"/>
         <v>899</v>
       </c>
       <c r="O133" s="10" t="s">
@@ -12329,6 +12448,7 @@
         <v>369</v>
       </c>
       <c r="E134" s="2">
+        <f t="shared" si="2"/>
         <v>857</v>
       </c>
       <c r="O134" s="10" t="s">
@@ -12352,6 +12472,7 @@
         <v>370</v>
       </c>
       <c r="E135" s="2">
+        <f t="shared" si="2"/>
         <v>705</v>
       </c>
       <c r="O135" s="10" t="s">
@@ -12375,6 +12496,7 @@
         <v>369</v>
       </c>
       <c r="E136" s="2">
+        <f t="shared" si="2"/>
         <v>2418</v>
       </c>
       <c r="O136" s="10" t="s">
@@ -12398,6 +12520,7 @@
         <v>370</v>
       </c>
       <c r="E137" s="2">
+        <f t="shared" si="2"/>
         <v>1706</v>
       </c>
       <c r="O137" s="10" t="s">
@@ -12421,6 +12544,7 @@
         <v>369</v>
       </c>
       <c r="E138" s="2">
+        <f t="shared" si="2"/>
         <v>1230</v>
       </c>
       <c r="O138" s="10" t="s">
@@ -12444,6 +12568,7 @@
         <v>370</v>
       </c>
       <c r="E139" s="2">
+        <f t="shared" si="2"/>
         <v>990</v>
       </c>
       <c r="O139" s="26" t="s">
@@ -12467,6 +12592,7 @@
         <v>369</v>
       </c>
       <c r="E140" s="2">
+        <f t="shared" si="2"/>
         <v>992</v>
       </c>
       <c r="O140" s="26" t="s">
@@ -12490,6 +12616,7 @@
         <v>370</v>
       </c>
       <c r="E141" s="2">
+        <f t="shared" si="2"/>
         <v>377</v>
       </c>
       <c r="O141" s="10" t="s">
@@ -12513,6 +12640,7 @@
         <v>369</v>
       </c>
       <c r="E142" s="2">
+        <f t="shared" si="2"/>
         <v>1076</v>
       </c>
       <c r="O142" s="10" t="s">
@@ -12536,6 +12664,7 @@
         <v>370</v>
       </c>
       <c r="E143" s="2">
+        <f t="shared" si="2"/>
         <v>803</v>
       </c>
       <c r="O143" s="10" t="s">
@@ -12559,6 +12688,7 @@
         <v>369</v>
       </c>
       <c r="E144" s="2">
+        <f t="shared" si="2"/>
         <v>1377</v>
       </c>
       <c r="O144" s="10" t="s">
@@ -12582,6 +12712,7 @@
         <v>370</v>
       </c>
       <c r="E145" s="2">
+        <f t="shared" si="2"/>
         <v>1864</v>
       </c>
       <c r="O145" s="10" t="s">
@@ -12601,7 +12732,8 @@
       <c r="D146" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E146" s="4">
+      <c r="E146" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O146" s="10" t="s">
@@ -12621,7 +12753,8 @@
       <c r="D147" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E147" s="4">
+      <c r="E147" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O147" s="26" t="s">
@@ -12641,7 +12774,8 @@
       <c r="D148" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E148" s="4">
+      <c r="E148" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O148" s="26" t="s">
@@ -12661,7 +12795,8 @@
       <c r="D149" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E149" s="4">
+      <c r="E149" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -12675,7 +12810,8 @@
       <c r="D150" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E150" s="4">
+      <c r="E150" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F150" s="2" t="s">
@@ -12692,7 +12828,8 @@
       <c r="D151" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E151" s="4">
+      <c r="E151" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F151" s="2" t="s">
@@ -12709,7 +12846,8 @@
       <c r="D152" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E152" s="4">
+      <c r="E152" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F152" s="2" t="s">
@@ -12726,7 +12864,8 @@
       <c r="D153" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E153" s="4">
+      <c r="E153" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F153" s="2" t="s">
@@ -12743,7 +12882,8 @@
       <c r="D154" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E154" s="4">
+      <c r="E154" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F154" s="2" t="s">
@@ -12760,7 +12900,8 @@
       <c r="D155" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E155" s="4">
+      <c r="E155" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F155" s="2" t="s">
@@ -12777,7 +12918,8 @@
       <c r="D156" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E156" s="4">
+      <c r="E156" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F156" s="2" t="s">
@@ -12794,7 +12936,8 @@
       <c r="D157" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E157" s="4">
+      <c r="E157" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F157" s="2" t="s">
@@ -12811,7 +12954,8 @@
       <c r="D158" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E158" s="4">
+      <c r="E158" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F158" s="2" t="s">
@@ -12828,7 +12972,8 @@
       <c r="D159" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E159" s="4">
+      <c r="E159" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F159" s="2" t="s">
@@ -12845,7 +12990,8 @@
       <c r="D160" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E160" s="4">
+      <c r="E160" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F160" s="2" t="s">
@@ -12862,7 +13008,8 @@
       <c r="D161" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E161" s="4">
+      <c r="E161" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F161" s="2" t="s">
@@ -12873,13 +13020,13 @@
       <c r="A162" s="2">
         <v>161</v>
       </c>
-      <c r="C162" s="4">
+      <c r="C162" s="30">
         <v>2025131</v>
       </c>
-      <c r="D162" s="4" t="s">
+      <c r="D162" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E162" s="4">
+      <c r="E162" s="30">
         <v>1040</v>
       </c>
       <c r="F162" s="2" t="s">
@@ -12890,13 +13037,13 @@
       <c r="A163" s="2">
         <v>162</v>
       </c>
-      <c r="C163" s="4">
+      <c r="C163" s="30">
         <v>2025131</v>
       </c>
-      <c r="D163" s="4" t="s">
+      <c r="D163" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E163" s="4">
+      <c r="E163" s="30">
         <v>1642</v>
       </c>
       <c r="F163" s="2" t="s">
@@ -12907,13 +13054,13 @@
       <c r="A164" s="2">
         <v>163</v>
       </c>
-      <c r="C164" s="4">
+      <c r="C164" s="30">
         <v>2025136</v>
       </c>
-      <c r="D164" s="4" t="s">
+      <c r="D164" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E164" s="4">
+      <c r="E164" s="30">
         <v>1396</v>
       </c>
       <c r="F164" s="2" t="s">
@@ -12924,13 +13071,13 @@
       <c r="A165" s="2">
         <v>164</v>
       </c>
-      <c r="C165" s="4">
+      <c r="C165" s="30">
         <v>2025136</v>
       </c>
-      <c r="D165" s="4" t="s">
+      <c r="D165" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E165" s="4">
+      <c r="E165" s="30">
         <v>916</v>
       </c>
       <c r="F165" s="2" t="s">
@@ -12941,13 +13088,13 @@
       <c r="A166" s="2">
         <v>165</v>
       </c>
-      <c r="C166" s="4">
+      <c r="C166" s="30">
         <v>2025111</v>
       </c>
-      <c r="D166" s="4" t="s">
+      <c r="D166" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E166" s="4">
+      <c r="E166" s="30">
         <v>1483</v>
       </c>
       <c r="F166" s="2" t="s">
@@ -12958,13 +13105,13 @@
       <c r="A167" s="2">
         <v>166</v>
       </c>
-      <c r="C167" s="4">
+      <c r="C167" s="30">
         <v>2025111</v>
       </c>
-      <c r="D167" s="4" t="s">
+      <c r="D167" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E167" s="4">
+      <c r="E167" s="30">
         <v>770</v>
       </c>
       <c r="F167" s="2" t="s">
@@ -12975,13 +13122,13 @@
       <c r="A168" s="2">
         <v>167</v>
       </c>
-      <c r="C168" s="4">
+      <c r="C168" s="30">
         <v>2025139</v>
       </c>
-      <c r="D168" s="4" t="s">
+      <c r="D168" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E168" s="4">
+      <c r="E168" s="30">
         <v>780</v>
       </c>
       <c r="F168" s="2" t="s">
@@ -12992,13 +13139,13 @@
       <c r="A169" s="2">
         <v>168</v>
       </c>
-      <c r="C169" s="4">
+      <c r="C169" s="30">
         <v>2025139</v>
       </c>
-      <c r="D169" s="4" t="s">
+      <c r="D169" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E169" s="4">
+      <c r="E169" s="30">
         <v>557</v>
       </c>
       <c r="F169" s="2" t="s">
@@ -13009,13 +13156,13 @@
       <c r="A170" s="2">
         <v>169</v>
       </c>
-      <c r="C170" s="4">
+      <c r="C170" s="30">
         <v>2025129</v>
       </c>
-      <c r="D170" s="4" t="s">
+      <c r="D170" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E170" s="4">
+      <c r="E170" s="30">
         <v>1517</v>
       </c>
       <c r="F170" s="2" t="s">
@@ -13026,13 +13173,13 @@
       <c r="A171" s="2">
         <v>170</v>
       </c>
-      <c r="C171" s="4">
+      <c r="C171" s="30">
         <v>2025129</v>
       </c>
-      <c r="D171" s="4" t="s">
+      <c r="D171" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E171" s="4">
+      <c r="E171" s="30">
         <v>811</v>
       </c>
       <c r="F171" s="2" t="s">
@@ -13043,13 +13190,13 @@
       <c r="A172" s="2">
         <v>171</v>
       </c>
-      <c r="C172" s="4">
+      <c r="C172" s="30">
         <v>2025112</v>
       </c>
-      <c r="D172" s="4" t="s">
+      <c r="D172" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E172" s="4">
+      <c r="E172" s="30">
         <v>718</v>
       </c>
       <c r="F172" s="2" t="s">
@@ -13060,13 +13207,13 @@
       <c r="A173" s="2">
         <v>172</v>
       </c>
-      <c r="C173" s="4">
+      <c r="C173" s="30">
         <v>2025112</v>
       </c>
-      <c r="D173" s="4" t="s">
+      <c r="D173" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E173" s="4">
+      <c r="E173" s="30">
         <v>512</v>
       </c>
       <c r="F173" s="2" t="s">
@@ -13077,13 +13224,13 @@
       <c r="A174" s="2">
         <v>173</v>
       </c>
-      <c r="C174" s="4">
+      <c r="C174" s="30">
         <v>2025090</v>
       </c>
-      <c r="D174" s="4" t="s">
+      <c r="D174" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E174" s="4">
+      <c r="E174" s="30">
         <v>1103</v>
       </c>
       <c r="F174" s="2" t="s">
@@ -13094,13 +13241,13 @@
       <c r="A175" s="2">
         <v>174</v>
       </c>
-      <c r="C175" s="4">
+      <c r="C175" s="30">
         <v>2025090</v>
       </c>
-      <c r="D175" s="4" t="s">
+      <c r="D175" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E175" s="4">
+      <c r="E175" s="30">
         <v>813</v>
       </c>
       <c r="F175" s="2" t="s">
@@ -13111,13 +13258,13 @@
       <c r="A176" s="2">
         <v>175</v>
       </c>
-      <c r="C176" s="4">
+      <c r="C176" s="30">
         <v>2025083</v>
       </c>
-      <c r="D176" s="4" t="s">
+      <c r="D176" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E176" s="4">
+      <c r="E176" s="30">
         <v>717</v>
       </c>
       <c r="F176" s="2" t="s">
@@ -13128,13 +13275,13 @@
       <c r="A177" s="2">
         <v>176</v>
       </c>
-      <c r="C177" s="4">
+      <c r="C177" s="30">
         <v>2025083</v>
       </c>
-      <c r="D177" s="4" t="s">
+      <c r="D177" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E177" s="4">
+      <c r="E177" s="30">
         <v>835</v>
       </c>
       <c r="F177" s="2" t="s">
@@ -13145,13 +13292,13 @@
       <c r="A178" s="2">
         <v>177</v>
       </c>
-      <c r="C178" s="4">
+      <c r="C178" s="30">
         <v>2025118</v>
       </c>
-      <c r="D178" s="4" t="s">
+      <c r="D178" s="30" t="s">
         <v>369</v>
       </c>
-      <c r="E178" s="4">
+      <c r="E178" s="30">
         <v>1378</v>
       </c>
       <c r="F178" s="2" t="s">
@@ -13159,13 +13306,13 @@
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C179" s="4">
+      <c r="C179" s="30">
         <v>2025118</v>
       </c>
-      <c r="D179" s="4" t="s">
+      <c r="D179" s="30" t="s">
         <v>370</v>
       </c>
-      <c r="E179" s="4">
+      <c r="E179" s="30">
         <v>929</v>
       </c>
       <c r="F179" s="2" t="s">

</xml_diff>